<commit_message>
updating specimen - morphosource
</commit_message>
<xml_diff>
--- a/Sample_data.xlsx
+++ b/Sample_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Document_UQAR\These\chapitre_2\Article\Repository\Raw_data_salamanders_modularity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{753304A8-0BE8-4375-AACA-57F87BF09064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF37345-E5DE-4677-BBB2-B77473938D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1369" uniqueCount="507">
   <si>
     <t>Family</t>
   </si>
@@ -1475,13 +1475,85 @@
   </si>
   <si>
     <t>Acronyms</t>
+  </si>
+  <si>
+    <t>000779270</t>
+  </si>
+  <si>
+    <t>URL Morphosource</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000779270?locale=en</t>
+  </si>
+  <si>
+    <t>000777739</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000777739?locale=en</t>
+  </si>
+  <si>
+    <t>000777734</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000777734?locale=en</t>
+  </si>
+  <si>
+    <t>000777729</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000777729?locale=en</t>
+  </si>
+  <si>
+    <t>000777724</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000777724?locale=en</t>
+  </si>
+  <si>
+    <t>000777717</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000777717?locale=en</t>
+  </si>
+  <si>
+    <t>000518007</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000518007?locale=en</t>
+  </si>
+  <si>
+    <t>000518299</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000518299?locale=en</t>
+  </si>
+  <si>
+    <t>000518335</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000518335?locale=en</t>
+  </si>
+  <si>
+    <t>000774866</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000774866?locale=en</t>
+  </si>
+  <si>
+    <t>000774878</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000774878/edit?locale=en</t>
+  </si>
+  <si>
+    <t>Upcoming</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1506,13 +1578,25 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1527,7 +1611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1542,6 +1626,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1766,7 +1861,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:R942"/>
+  <dimension ref="A1:S942"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.140625" customWidth="1"/>
@@ -1781,10 +1876,11 @@
     <col min="15" max="15" width="27" customWidth="1"/>
     <col min="16" max="16" width="35.42578125" customWidth="1"/>
     <col min="17" max="17" width="13.85546875" customWidth="1"/>
-    <col min="18" max="18" width="34.7109375" customWidth="1"/>
+    <col min="18" max="18" width="34.7109375" style="7" customWidth="1"/>
+    <col min="19" max="19" width="32.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1836,11 +1932,14 @@
       <c r="Q1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="6" t="s">
         <v>401</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S1" s="4" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>23</v>
       </c>
@@ -1888,8 +1987,11 @@
       </c>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
-    </row>
-    <row r="3" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R2" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>23</v>
       </c>
@@ -1941,8 +2043,11 @@
       <c r="Q3" s="3" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R3" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>23</v>
       </c>
@@ -1994,8 +2099,11 @@
       <c r="Q4" s="3" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R4" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
@@ -2039,8 +2147,11 @@
       <c r="Q5" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R5" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>23</v>
       </c>
@@ -2092,8 +2203,11 @@
       <c r="Q6" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R6" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>23</v>
       </c>
@@ -2145,8 +2259,11 @@
       <c r="Q7" s="3" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R7" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>23</v>
       </c>
@@ -2194,8 +2311,11 @@
       </c>
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
-    </row>
-    <row r="9" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R8" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>299</v>
       </c>
@@ -2241,8 +2361,11 @@
       <c r="Q9" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="10" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R9" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>33</v>
       </c>
@@ -2292,8 +2415,11 @@
       <c r="Q10" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R10" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>33</v>
       </c>
@@ -2343,8 +2469,11 @@
       <c r="Q11" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="12" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R11" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>33</v>
       </c>
@@ -2394,8 +2523,11 @@
       <c r="Q12" s="3" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R12" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>33</v>
       </c>
@@ -2445,8 +2577,11 @@
       <c r="Q13" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R13" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>33</v>
       </c>
@@ -2496,15 +2631,18 @@
       <c r="Q14" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="15" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R14" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="8" t="s">
         <v>203</v>
       </c>
       <c r="D15" s="3" t="s">
@@ -2545,15 +2683,21 @@
       </c>
       <c r="P15" s="3"/>
       <c r="Q15" s="3"/>
-    </row>
-    <row r="16" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R15" s="7" t="s">
+        <v>504</v>
+      </c>
+      <c r="S15" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="8" t="s">
         <v>203</v>
       </c>
       <c r="D16" s="3" t="s">
@@ -2594,15 +2738,21 @@
       </c>
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
-    </row>
-    <row r="17" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R16" s="7" t="s">
+        <v>502</v>
+      </c>
+      <c r="S16" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="8" t="s">
         <v>335</v>
       </c>
       <c r="D17" s="3" t="s">
@@ -2645,8 +2795,14 @@
       <c r="Q17" s="3" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R17" s="7" t="s">
+        <v>500</v>
+      </c>
+      <c r="S17" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>33</v>
       </c>
@@ -2696,8 +2852,11 @@
       <c r="Q18" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="19" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R18" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>33</v>
       </c>
@@ -2747,8 +2906,11 @@
       <c r="Q19" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="20" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R19" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>33</v>
       </c>
@@ -2798,8 +2960,11 @@
       <c r="Q20" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R20" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>33</v>
       </c>
@@ -2851,8 +3016,11 @@
       <c r="Q21" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R21" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>33</v>
       </c>
@@ -2904,8 +3072,11 @@
       <c r="Q22" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R22" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>33</v>
       </c>
@@ -2955,8 +3126,11 @@
       <c r="Q23" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R23" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>33</v>
       </c>
@@ -3008,8 +3182,11 @@
       <c r="Q24" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R24" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
         <v>33</v>
       </c>
@@ -3061,8 +3238,11 @@
       <c r="Q25" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R25" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>33</v>
       </c>
@@ -3114,8 +3294,11 @@
       <c r="Q26" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R26" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
         <v>33</v>
       </c>
@@ -3167,8 +3350,11 @@
       <c r="Q27" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R27" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>33</v>
       </c>
@@ -3218,8 +3404,11 @@
       <c r="Q28" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="29" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R28" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>304</v>
       </c>
@@ -3265,8 +3454,11 @@
       <c r="Q29" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="30" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R29" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
         <v>33</v>
       </c>
@@ -3318,8 +3510,11 @@
       <c r="Q30" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="31" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R30" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
         <v>65</v>
       </c>
@@ -3369,8 +3564,11 @@
       <c r="Q31" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="32" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R31" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>33</v>
       </c>
@@ -3422,8 +3620,11 @@
       <c r="Q32" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="33" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R32" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
         <v>33</v>
       </c>
@@ -3473,8 +3674,11 @@
       <c r="Q33" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="34" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R33" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
         <v>33</v>
       </c>
@@ -3524,15 +3728,18 @@
       <c r="Q34" s="3" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="35" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R34" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="8" t="s">
         <v>341</v>
       </c>
       <c r="D35" s="3" t="s">
@@ -3575,8 +3782,14 @@
       <c r="Q35" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="36" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R35" s="7" t="s">
+        <v>498</v>
+      </c>
+      <c r="S35" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>308</v>
       </c>
@@ -3620,8 +3833,11 @@
       <c r="Q36" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="37" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R36" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
         <v>33</v>
       </c>
@@ -3671,8 +3887,11 @@
       <c r="Q37" s="3" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="38" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R37" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
         <v>33</v>
       </c>
@@ -3722,8 +3941,11 @@
       <c r="Q38" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="39" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R38" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
         <v>33</v>
       </c>
@@ -3773,8 +3995,11 @@
       <c r="Q39" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="40" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R39" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
         <v>33</v>
       </c>
@@ -3824,8 +4049,11 @@
       <c r="Q40" s="3" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="41" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R40" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
         <v>33</v>
       </c>
@@ -3875,8 +4103,11 @@
       <c r="Q41" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="42" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R41" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
         <v>33</v>
       </c>
@@ -3926,8 +4157,11 @@
       <c r="Q42" s="3" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="43" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R42" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
         <v>33</v>
       </c>
@@ -3979,15 +4213,18 @@
       <c r="Q43" s="3" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="44" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R43" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="8" t="s">
         <v>74</v>
       </c>
       <c r="D44" s="3" t="s">
@@ -4028,8 +4265,14 @@
       </c>
       <c r="P44" s="3"/>
       <c r="Q44" s="3"/>
-    </row>
-    <row r="45" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R44" s="7" t="s">
+        <v>494</v>
+      </c>
+      <c r="S44" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
         <v>33</v>
       </c>
@@ -4079,8 +4322,11 @@
       <c r="Q45" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="46" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R45" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
         <v>51</v>
       </c>
@@ -4132,8 +4378,11 @@
       <c r="Q46" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="47" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R46" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
         <v>51</v>
       </c>
@@ -4177,8 +4426,11 @@
       <c r="Q47" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="48" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R47" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
         <v>51</v>
       </c>
@@ -4230,8 +4482,11 @@
       <c r="Q48" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="49" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R48" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
         <v>51</v>
       </c>
@@ -4283,8 +4538,11 @@
       <c r="Q49" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="50" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R49" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>51</v>
       </c>
@@ -4336,8 +4594,11 @@
       <c r="Q50" s="3" t="s">
         <v>399</v>
       </c>
-    </row>
-    <row r="51" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R50" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
         <v>65</v>
       </c>
@@ -4387,15 +4648,18 @@
       <c r="Q51" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="52" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R51" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C52" s="8" t="s">
         <v>39</v>
       </c>
       <c r="D52" s="3" t="s">
@@ -4436,15 +4700,21 @@
       </c>
       <c r="P52" s="3"/>
       <c r="Q52" s="3"/>
-    </row>
-    <row r="53" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R52" s="9" t="s">
+        <v>483</v>
+      </c>
+      <c r="S52" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C53" s="8" t="s">
         <v>39</v>
       </c>
       <c r="D53" s="3" t="s">
@@ -4485,8 +4755,14 @@
       </c>
       <c r="P53" s="3"/>
       <c r="Q53" s="3"/>
-    </row>
-    <row r="54" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R53" s="7" t="s">
+        <v>492</v>
+      </c>
+      <c r="S53" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
         <v>33</v>
       </c>
@@ -4538,15 +4814,18 @@
       <c r="Q54" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="55" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R54" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="C55" s="8" t="s">
         <v>78</v>
       </c>
       <c r="D55" s="3" t="s">
@@ -4587,8 +4866,14 @@
       </c>
       <c r="P55" s="3"/>
       <c r="Q55" s="3"/>
-    </row>
-    <row r="56" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R55" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="S55" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
         <v>65</v>
       </c>
@@ -4638,8 +4923,11 @@
       <c r="Q56" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="57" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R56" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="57" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
         <v>16</v>
       </c>
@@ -4691,8 +4979,11 @@
       <c r="Q57" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="58" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R57" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="58" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
         <v>16</v>
       </c>
@@ -4744,8 +5035,11 @@
       <c r="Q58" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="59" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R58" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="59" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
         <v>65</v>
       </c>
@@ -4797,8 +5091,11 @@
       <c r="Q59" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="60" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R59" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="60" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
         <v>65</v>
       </c>
@@ -4850,8 +5147,11 @@
       <c r="Q60" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="61" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R60" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
         <v>33</v>
       </c>
@@ -4901,15 +5201,18 @@
       <c r="Q61" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="62" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R61" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="62" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="C62" s="8" t="s">
         <v>80</v>
       </c>
       <c r="D62" s="3" t="s">
@@ -4950,8 +5253,14 @@
       </c>
       <c r="P62" s="3"/>
       <c r="Q62" s="3"/>
-    </row>
-    <row r="63" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R62" s="7" t="s">
+        <v>490</v>
+      </c>
+      <c r="S62" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="63" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
         <v>33</v>
       </c>
@@ -5001,8 +5310,11 @@
       <c r="Q63" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="64" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R63" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="64" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
         <v>51</v>
       </c>
@@ -5054,8 +5366,11 @@
       <c r="Q64" s="3" t="s">
         <v>334</v>
       </c>
-    </row>
-    <row r="65" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R64" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="65" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>65</v>
       </c>
@@ -5107,8 +5422,11 @@
       <c r="Q65" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="66" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R65" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="66" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
         <v>33</v>
       </c>
@@ -5160,8 +5478,11 @@
       <c r="Q66" s="3" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="67" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R66" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="67" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
         <v>33</v>
       </c>
@@ -5211,8 +5532,11 @@
       <c r="Q67" s="3" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="68" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R67" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="68" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
         <v>33</v>
       </c>
@@ -5262,8 +5586,11 @@
       <c r="Q68" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="69" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R68" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="69" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
         <v>33</v>
       </c>
@@ -5313,8 +5640,11 @@
       <c r="Q69" s="3" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="70" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R69" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="70" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
         <v>33</v>
       </c>
@@ -5358,8 +5688,11 @@
       <c r="Q70" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="71" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R70" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="71" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
         <v>33</v>
       </c>
@@ -5405,8 +5738,11 @@
       <c r="Q71" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="72" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R71" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="72" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
         <v>33</v>
       </c>
@@ -5452,8 +5788,11 @@
       <c r="Q72" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="73" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R72" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="73" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="s">
         <v>110</v>
       </c>
@@ -5497,8 +5836,11 @@
       <c r="Q73" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="74" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R73" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="74" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
         <v>33</v>
       </c>
@@ -5548,8 +5890,11 @@
       <c r="Q74" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="75" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R74" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="75" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
         <v>33</v>
       </c>
@@ -5599,8 +5944,11 @@
       <c r="Q75" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="76" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R75" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="76" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
         <v>33</v>
       </c>
@@ -5650,8 +5998,11 @@
       <c r="Q76" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="77" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R76" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="77" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="3" t="s">
         <v>191</v>
       </c>
@@ -5701,8 +6052,11 @@
       <c r="Q77" s="3" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="78" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R77" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="78" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="3" t="s">
         <v>65</v>
       </c>
@@ -5752,8 +6106,11 @@
       <c r="Q78" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="79" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R78" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="79" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="3" t="s">
         <v>51</v>
       </c>
@@ -5805,8 +6162,11 @@
       <c r="Q79" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="80" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R79" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="80" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="3" t="s">
         <v>110</v>
       </c>
@@ -5852,8 +6212,11 @@
       <c r="Q80" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="81" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R80" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="81" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="3" t="s">
         <v>65</v>
       </c>
@@ -5905,15 +6268,18 @@
       <c r="Q81" s="3" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="82" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R81" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="82" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B82" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C82" s="3" t="s">
+      <c r="C82" s="8" t="s">
         <v>83</v>
       </c>
       <c r="D82" s="3" t="s">
@@ -5954,8 +6320,14 @@
       </c>
       <c r="P82" s="3"/>
       <c r="Q82" s="3"/>
-    </row>
-    <row r="83" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R82" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="S82" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="83" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3" t="s">
         <v>33</v>
       </c>
@@ -6007,8 +6379,11 @@
       <c r="Q83" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="84" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R83" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="84" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3" t="s">
         <v>33</v>
       </c>
@@ -6060,8 +6435,11 @@
       <c r="Q84" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="85" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R84" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="85" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="3" t="s">
         <v>33</v>
       </c>
@@ -6111,8 +6489,11 @@
       <c r="Q85" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="86" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R85" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="86" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
         <v>33</v>
       </c>
@@ -6164,8 +6545,11 @@
       <c r="Q86" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="87" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R86" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="87" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="s">
         <v>33</v>
       </c>
@@ -6215,8 +6599,11 @@
       <c r="Q87" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="88" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R87" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="88" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="3" t="s">
         <v>65</v>
       </c>
@@ -6266,8 +6653,11 @@
       <c r="Q88" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="89" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R88" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="89" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
         <v>65</v>
       </c>
@@ -6319,15 +6709,18 @@
       <c r="Q89" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="90" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R89" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="90" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B90" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="C90" s="3" t="s">
+      <c r="C90" s="8" t="s">
         <v>344</v>
       </c>
       <c r="D90" s="3" t="s">
@@ -6372,13 +6765,19 @@
       <c r="Q90" s="3" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="91" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="92" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="93" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="94" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="95" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="96" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="R90" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="S90" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="91" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="92" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="93" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="94" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="95" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="96" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
added several specimens -morphosource
</commit_message>
<xml_diff>
--- a/Sample_data.xlsx
+++ b/Sample_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Document_UQAR\These\chapitre_2\Article\Repository\Raw_data_salamanders_modularity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF37345-E5DE-4677-BBB2-B77473938D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0618BBE-8B69-4E82-9B93-F596652C98DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1369" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1380" uniqueCount="529">
   <si>
     <t>Family</t>
   </si>
@@ -1547,6 +1547,72 @@
   </si>
   <si>
     <t>Upcoming</t>
+  </si>
+  <si>
+    <t>000386438</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000386438?locale=en</t>
+  </si>
+  <si>
+    <t>000067236</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000067236?locale=en</t>
+  </si>
+  <si>
+    <t>000159507</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000159507?locale=en</t>
+  </si>
+  <si>
+    <t>000133947</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000133947?locale=en</t>
+  </si>
+  <si>
+    <t>000433298</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000433298?locale=en</t>
+  </si>
+  <si>
+    <t>000432922</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000432922?locale=en</t>
+  </si>
+  <si>
+    <t>000433303</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000433303?locale=en</t>
+  </si>
+  <si>
+    <t>000364327</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000364327?locale=en</t>
+  </si>
+  <si>
+    <t>000857282</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000857282?locale=en</t>
+  </si>
+  <si>
+    <t>000857293</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000857293?locale=en</t>
+  </si>
+  <si>
+    <t>000857303</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000857303?locale=en</t>
   </si>
 </sst>
 </file>
@@ -1946,7 +2012,7 @@
       <c r="B2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="8" t="s">
         <v>108</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -1988,7 +2054,10 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="10" t="s">
-        <v>506</v>
+        <v>527</v>
+      </c>
+      <c r="S2" t="s">
+        <v>528</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2322,7 +2391,7 @@
       <c r="B9" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="8" t="s">
         <v>301</v>
       </c>
       <c r="D9" s="3" t="s">
@@ -2362,7 +2431,10 @@
         <v>21</v>
       </c>
       <c r="R9" s="10" t="s">
-        <v>506</v>
+        <v>507</v>
+      </c>
+      <c r="S9" t="s">
+        <v>508</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2534,7 +2606,7 @@
       <c r="B13" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="8" t="s">
         <v>212</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -2578,7 +2650,10 @@
         <v>21</v>
       </c>
       <c r="R13" s="10" t="s">
-        <v>506</v>
+        <v>523</v>
+      </c>
+      <c r="S13" t="s">
+        <v>524</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2588,7 +2663,7 @@
       <c r="B14" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="8" t="s">
         <v>215</v>
       </c>
       <c r="D14" s="3" t="s">
@@ -2632,7 +2707,10 @@
         <v>21</v>
       </c>
       <c r="R14" s="10" t="s">
-        <v>506</v>
+        <v>525</v>
+      </c>
+      <c r="S14" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3415,7 +3493,7 @@
       <c r="B29" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="8" t="s">
         <v>306</v>
       </c>
       <c r="D29" s="3" t="s">
@@ -3455,7 +3533,10 @@
         <v>21</v>
       </c>
       <c r="R29" s="10" t="s">
-        <v>506</v>
+        <v>509</v>
+      </c>
+      <c r="S29" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="30" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3796,7 +3877,7 @@
       <c r="B36" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="8" t="s">
         <v>310</v>
       </c>
       <c r="D36" s="3" t="s">
@@ -3834,7 +3915,10 @@
         <v>21</v>
       </c>
       <c r="R36" s="10" t="s">
-        <v>506</v>
+        <v>511</v>
+      </c>
+      <c r="S36" t="s">
+        <v>512</v>
       </c>
     </row>
     <row r="37" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4389,7 +4473,7 @@
       <c r="B47" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C47" s="8" t="s">
         <v>312</v>
       </c>
       <c r="D47" s="3" t="s">
@@ -4427,7 +4511,10 @@
         <v>21</v>
       </c>
       <c r="R47" s="10" t="s">
-        <v>506</v>
+        <v>513</v>
+      </c>
+      <c r="S47" t="s">
+        <v>514</v>
       </c>
     </row>
     <row r="48" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5370,7 +5457,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="65" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>65</v>
       </c>
@@ -5426,7 +5513,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="66" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
         <v>33</v>
       </c>
@@ -5482,7 +5569,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
         <v>33</v>
       </c>
@@ -5536,7 +5623,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
         <v>33</v>
       </c>
@@ -5590,7 +5677,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="69" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
         <v>33</v>
       </c>
@@ -5644,14 +5731,14 @@
         <v>506</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C70" s="3" t="s">
+      <c r="C70" s="8" t="s">
         <v>296</v>
       </c>
       <c r="D70" s="3" t="s">
@@ -5689,17 +5776,20 @@
         <v>21</v>
       </c>
       <c r="R70" s="10" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="71" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>515</v>
+      </c>
+      <c r="S70" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="71" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C71" s="3" t="s">
+      <c r="C71" s="8" t="s">
         <v>67</v>
       </c>
       <c r="D71" s="3" t="s">
@@ -5739,17 +5829,20 @@
         <v>21</v>
       </c>
       <c r="R71" s="10" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="72" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>517</v>
+      </c>
+      <c r="S71" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="72" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C72" s="3" t="s">
+      <c r="C72" s="8" t="s">
         <v>67</v>
       </c>
       <c r="D72" s="3" t="s">
@@ -5789,10 +5882,13 @@
         <v>21</v>
       </c>
       <c r="R72" s="10" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="73" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>519</v>
+      </c>
+      <c r="S72" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="73" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="s">
         <v>110</v>
       </c>
@@ -5840,7 +5936,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
         <v>33</v>
       </c>
@@ -5894,7 +5990,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
         <v>33</v>
       </c>
@@ -5948,7 +6044,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="76" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
         <v>33</v>
       </c>
@@ -6002,7 +6098,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="77" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="3" t="s">
         <v>191</v>
       </c>
@@ -6056,7 +6152,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="78" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="3" t="s">
         <v>65</v>
       </c>
@@ -6110,7 +6206,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="79" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="3" t="s">
         <v>51</v>
       </c>
@@ -6166,14 +6262,14 @@
         <v>506</v>
       </c>
     </row>
-    <row r="80" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="3" t="s">
         <v>110</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="C80" s="3" t="s">
+      <c r="C80" s="8" t="s">
         <v>112</v>
       </c>
       <c r="D80" s="3" t="s">
@@ -6213,7 +6309,10 @@
         <v>21</v>
       </c>
       <c r="R80" s="10" t="s">
-        <v>506</v>
+        <v>521</v>
+      </c>
+      <c r="S80" t="s">
+        <v>522</v>
       </c>
     </row>
     <row r="81" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
adding specimens on morphosource
</commit_message>
<xml_diff>
--- a/Sample_data.xlsx
+++ b/Sample_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Document_UQAR\These\chapitre_2\Article\Repository\Raw_data_salamanders_modularity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44526809-09E3-40AF-8B45-86548A5112BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C426552-BEF6-443A-B2B6-00BC895FFEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="551">
   <si>
     <t>Family</t>
   </si>
@@ -1637,6 +1637,48 @@
   </si>
   <si>
     <t>https://www.morphosource.org/concern/media/000857537?locale=en</t>
+  </si>
+  <si>
+    <t>000859397</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859397?locale=en</t>
+  </si>
+  <si>
+    <t>000859402</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859402?locale=en</t>
+  </si>
+  <si>
+    <t>000859407</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859407?locale=en</t>
+  </si>
+  <si>
+    <t>000859414</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859414?locale=en</t>
+  </si>
+  <si>
+    <t>000859426</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859426?locale=en</t>
+  </si>
+  <si>
+    <t>000859433</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859433?locale=en</t>
+  </si>
+  <si>
+    <t>000859442</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859442?locale=en</t>
   </si>
 </sst>
 </file>
@@ -1675,12 +1717,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1695,7 +1743,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1718,6 +1766,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2030,7 +2081,7 @@
       <c r="B2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="3" t="s">
         <v>108</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -2085,7 +2136,7 @@
       <c r="B3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="3" t="s">
         <v>120</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -2141,7 +2192,7 @@
       <c r="B4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="3" t="s">
         <v>124</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -2197,7 +2248,7 @@
       <c r="B5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="3" t="s">
         <v>113</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -2243,7 +2294,7 @@
       <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="3" t="s">
         <v>128</v>
       </c>
       <c r="D6" s="3" t="s">
@@ -2299,7 +2350,7 @@
       <c r="B7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="3" t="s">
         <v>130</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -2355,7 +2406,7 @@
       <c r="B8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="3" t="s">
         <v>70</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -2407,7 +2458,7 @@
       <c r="B9" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="3" t="s">
         <v>301</v>
       </c>
       <c r="D9" s="3" t="s">
@@ -2460,7 +2511,7 @@
       <c r="B10" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="3" t="s">
         <v>142</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -2514,7 +2565,7 @@
       <c r="B11" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="3" t="s">
         <v>136</v>
       </c>
       <c r="D11" s="3" t="s">
@@ -2568,7 +2619,7 @@
       <c r="B12" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="3" t="s">
         <v>137</v>
       </c>
       <c r="D12" s="3" t="s">
@@ -2622,7 +2673,7 @@
       <c r="B13" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="3" t="s">
         <v>212</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -2679,7 +2730,7 @@
       <c r="B14" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="3" t="s">
         <v>215</v>
       </c>
       <c r="D14" s="3" t="s">
@@ -2736,7 +2787,7 @@
       <c r="B15" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="3" t="s">
         <v>203</v>
       </c>
       <c r="D15" s="3" t="s">
@@ -2791,7 +2842,7 @@
       <c r="B16" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="3" t="s">
         <v>203</v>
       </c>
       <c r="D16" s="3" t="s">
@@ -2846,7 +2897,7 @@
       <c r="B17" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="3" t="s">
         <v>335</v>
       </c>
       <c r="D17" s="3" t="s">
@@ -2903,7 +2954,7 @@
       <c r="B18" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="3" t="s">
         <v>235</v>
       </c>
       <c r="D18" s="3" t="s">
@@ -2960,7 +3011,7 @@
       <c r="B19" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="3" t="s">
         <v>239</v>
       </c>
       <c r="D19" s="3" t="s">
@@ -3017,7 +3068,7 @@
       <c r="B20" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="3" t="s">
         <v>228</v>
       </c>
       <c r="D20" s="3" t="s">
@@ -3074,7 +3125,7 @@
       <c r="B21" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="3" t="s">
         <v>243</v>
       </c>
       <c r="D21" s="3" t="s">
@@ -3133,7 +3184,7 @@
       <c r="B22" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="11" t="s">
         <v>225</v>
       </c>
       <c r="D22" s="3" t="s">
@@ -3179,7 +3230,10 @@
         <v>21</v>
       </c>
       <c r="R22" s="9" t="s">
-        <v>506</v>
+        <v>539</v>
+      </c>
+      <c r="S22" t="s">
+        <v>540</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3189,7 +3243,7 @@
       <c r="B23" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="11" t="s">
         <v>222</v>
       </c>
       <c r="D23" s="3" t="s">
@@ -3233,7 +3287,10 @@
         <v>21</v>
       </c>
       <c r="R23" s="9" t="s">
-        <v>506</v>
+        <v>537</v>
+      </c>
+      <c r="S23" t="s">
+        <v>538</v>
       </c>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3243,7 +3300,7 @@
       <c r="B24" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="11" t="s">
         <v>218</v>
       </c>
       <c r="D24" s="3" t="s">
@@ -3289,7 +3346,10 @@
         <v>21</v>
       </c>
       <c r="R24" s="9" t="s">
-        <v>506</v>
+        <v>547</v>
+      </c>
+      <c r="S24" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3299,7 +3359,7 @@
       <c r="B25" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="11" t="s">
         <v>230</v>
       </c>
       <c r="D25" s="3" t="s">
@@ -3345,7 +3405,10 @@
         <v>21</v>
       </c>
       <c r="R25" s="9" t="s">
-        <v>506</v>
+        <v>543</v>
+      </c>
+      <c r="S25" t="s">
+        <v>544</v>
       </c>
     </row>
     <row r="26" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3355,7 +3418,7 @@
       <c r="B26" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="11" t="s">
         <v>230</v>
       </c>
       <c r="D26" s="3" t="s">
@@ -3401,7 +3464,10 @@
         <v>21</v>
       </c>
       <c r="R26" s="9" t="s">
-        <v>506</v>
+        <v>545</v>
+      </c>
+      <c r="S26" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="27" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3457,7 +3523,10 @@
         <v>21</v>
       </c>
       <c r="R27" s="9" t="s">
-        <v>506</v>
+        <v>549</v>
+      </c>
+      <c r="S27" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3467,7 +3536,7 @@
       <c r="B28" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="11" t="s">
         <v>246</v>
       </c>
       <c r="D28" s="3" t="s">
@@ -3511,7 +3580,10 @@
         <v>21</v>
       </c>
       <c r="R28" s="9" t="s">
-        <v>506</v>
+        <v>541</v>
+      </c>
+      <c r="S28" t="s">
+        <v>542</v>
       </c>
     </row>
     <row r="29" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3521,7 +3593,7 @@
       <c r="B29" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="3" t="s">
         <v>306</v>
       </c>
       <c r="D29" s="3" t="s">
@@ -3574,7 +3646,7 @@
       <c r="B30" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="3" t="s">
         <v>315</v>
       </c>
       <c r="D30" s="3" t="s">
@@ -3630,7 +3702,7 @@
       <c r="B31" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="3" t="s">
         <v>146</v>
       </c>
       <c r="D31" s="3" t="s">
@@ -3684,7 +3756,7 @@
       <c r="B32" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="3" t="s">
         <v>318</v>
       </c>
       <c r="D32" s="3" t="s">
@@ -3740,7 +3812,7 @@
       <c r="B33" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="3" t="s">
         <v>147</v>
       </c>
       <c r="D33" s="3" t="s">
@@ -3794,7 +3866,7 @@
       <c r="B34" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C34" s="3" t="s">
         <v>148</v>
       </c>
       <c r="D34" s="3" t="s">
@@ -3848,7 +3920,7 @@
       <c r="B35" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="C35" s="3" t="s">
         <v>341</v>
       </c>
       <c r="D35" s="3" t="s">
@@ -3905,7 +3977,7 @@
       <c r="B36" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="C36" s="3" t="s">
         <v>310</v>
       </c>
       <c r="D36" s="3" t="s">
@@ -3956,7 +4028,7 @@
       <c r="B37" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="C37" s="3" t="s">
         <v>153</v>
       </c>
       <c r="D37" s="3" t="s">
@@ -4010,7 +4082,7 @@
       <c r="B38" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C38" s="10" t="s">
+      <c r="C38" s="3" t="s">
         <v>158</v>
       </c>
       <c r="D38" s="3" t="s">
@@ -4064,7 +4136,7 @@
       <c r="B39" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="3" t="s">
         <v>249</v>
       </c>
       <c r="D39" s="3" t="s">
@@ -4118,7 +4190,7 @@
       <c r="B40" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="3" t="s">
         <v>161</v>
       </c>
       <c r="D40" s="3" t="s">
@@ -4172,7 +4244,7 @@
       <c r="B41" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="3" t="s">
         <v>252</v>
       </c>
       <c r="D41" s="3" t="s">
@@ -4226,7 +4298,7 @@
       <c r="B42" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="3" t="s">
         <v>166</v>
       </c>
       <c r="D42" s="3" t="s">
@@ -4280,7 +4352,7 @@
       <c r="B43" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="C43" s="10" t="s">
+      <c r="C43" s="3" t="s">
         <v>171</v>
       </c>
       <c r="D43" s="3" t="s">
@@ -4336,7 +4408,7 @@
       <c r="B44" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="C44" s="3" t="s">
         <v>74</v>
       </c>
       <c r="D44" s="3" t="s">
@@ -4391,7 +4463,7 @@
       <c r="B45" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C45" s="10" t="s">
+      <c r="C45" s="3" t="s">
         <v>322</v>
       </c>
       <c r="D45" s="3" t="s">
@@ -4445,7 +4517,7 @@
       <c r="B46" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C46" s="10" t="s">
+      <c r="C46" s="3" t="s">
         <v>255</v>
       </c>
       <c r="D46" s="3" t="s">
@@ -4501,7 +4573,7 @@
       <c r="B47" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="C47" s="3" t="s">
         <v>312</v>
       </c>
       <c r="D47" s="3" t="s">
@@ -4552,7 +4624,7 @@
       <c r="B48" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C48" s="10" t="s">
+      <c r="C48" s="3" t="s">
         <v>387</v>
       </c>
       <c r="D48" s="3" t="s">
@@ -4608,7 +4680,7 @@
       <c r="B49" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C49" s="10" t="s">
+      <c r="C49" s="3" t="s">
         <v>259</v>
       </c>
       <c r="D49" s="3" t="s">
@@ -4664,7 +4736,7 @@
       <c r="B50" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C50" s="10" t="s">
+      <c r="C50" s="3" t="s">
         <v>396</v>
       </c>
       <c r="D50" s="3" t="s">
@@ -4720,7 +4792,7 @@
       <c r="B51" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="C51" s="10" t="s">
+      <c r="C51" s="3" t="s">
         <v>177</v>
       </c>
       <c r="D51" s="3" t="s">
@@ -4774,7 +4846,7 @@
       <c r="B52" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C52" s="10" t="s">
+      <c r="C52" s="3" t="s">
         <v>39</v>
       </c>
       <c r="D52" s="3" t="s">
@@ -4829,7 +4901,7 @@
       <c r="B53" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C53" s="10" t="s">
+      <c r="C53" s="3" t="s">
         <v>39</v>
       </c>
       <c r="D53" s="3" t="s">
@@ -4884,7 +4956,7 @@
       <c r="B54" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C54" s="10" t="s">
+      <c r="C54" s="3" t="s">
         <v>39</v>
       </c>
       <c r="D54" s="3" t="s">
@@ -4940,7 +5012,7 @@
       <c r="B55" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C55" s="10" t="s">
+      <c r="C55" s="3" t="s">
         <v>78</v>
       </c>
       <c r="D55" s="3" t="s">
@@ -4995,7 +5067,7 @@
       <c r="B56" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="C56" s="10" t="s">
+      <c r="C56" s="3" t="s">
         <v>326</v>
       </c>
       <c r="D56" s="3" t="s">
@@ -5049,7 +5121,7 @@
       <c r="B57" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C57" s="10" t="s">
+      <c r="C57" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D57" s="3" t="s">
@@ -5105,7 +5177,7 @@
       <c r="B58" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C58" s="10" t="s">
+      <c r="C58" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D58" s="3" t="s">
@@ -5161,7 +5233,7 @@
       <c r="B59" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="C59" s="10" t="s">
+      <c r="C59" s="3" t="s">
         <v>353</v>
       </c>
       <c r="D59" s="3" t="s">
@@ -5217,7 +5289,7 @@
       <c r="B60" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="C60" s="10" t="s">
+      <c r="C60" s="3" t="s">
         <v>353</v>
       </c>
       <c r="D60" s="3" t="s">
@@ -5273,7 +5345,7 @@
       <c r="B61" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C61" s="10" t="s">
+      <c r="C61" s="3" t="s">
         <v>266</v>
       </c>
       <c r="D61" s="3" t="s">
@@ -5327,7 +5399,7 @@
       <c r="B62" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C62" s="10" t="s">
+      <c r="C62" s="3" t="s">
         <v>80</v>
       </c>
       <c r="D62" s="3" t="s">
@@ -5382,7 +5454,7 @@
       <c r="B63" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C63" s="10" t="s">
+      <c r="C63" s="3" t="s">
         <v>267</v>
       </c>
       <c r="D63" s="3" t="s">
@@ -5436,7 +5508,7 @@
       <c r="B64" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C64" s="10" t="s">
+      <c r="C64" s="3" t="s">
         <v>331</v>
       </c>
       <c r="D64" s="3" t="s">
@@ -5492,7 +5564,7 @@
       <c r="B65" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C65" s="10" t="s">
+      <c r="C65" s="3" t="s">
         <v>117</v>
       </c>
       <c r="D65" s="3" t="s">
@@ -5548,7 +5620,7 @@
       <c r="B66" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C66" s="10" t="s">
+      <c r="C66" s="3" t="s">
         <v>102</v>
       </c>
       <c r="D66" s="3" t="s">
@@ -5604,7 +5676,7 @@
       <c r="B67" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C67" s="10" t="s">
+      <c r="C67" s="3" t="s">
         <v>184</v>
       </c>
       <c r="D67" s="3" t="s">
@@ -5658,7 +5730,7 @@
       <c r="B68" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C68" s="10" t="s">
+      <c r="C68" s="3" t="s">
         <v>182</v>
       </c>
       <c r="D68" s="3" t="s">
@@ -5712,7 +5784,7 @@
       <c r="B69" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C69" s="10" t="s">
+      <c r="C69" s="3" t="s">
         <v>178</v>
       </c>
       <c r="D69" s="3" t="s">
@@ -5766,7 +5838,7 @@
       <c r="B70" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C70" s="10" t="s">
+      <c r="C70" s="3" t="s">
         <v>296</v>
       </c>
       <c r="D70" s="3" t="s">
@@ -5817,7 +5889,7 @@
       <c r="B71" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C71" s="10" t="s">
+      <c r="C71" s="3" t="s">
         <v>67</v>
       </c>
       <c r="D71" s="3" t="s">
@@ -5870,7 +5942,7 @@
       <c r="B72" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C72" s="10" t="s">
+      <c r="C72" s="3" t="s">
         <v>67</v>
       </c>
       <c r="D72" s="3" t="s">
@@ -5923,7 +5995,7 @@
       <c r="B73" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C73" s="10" t="s">
+      <c r="C73" s="3" t="s">
         <v>115</v>
       </c>
       <c r="D73" s="3" t="s">
@@ -5969,7 +6041,7 @@
       <c r="B74" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C74" s="10" t="s">
+      <c r="C74" s="3" t="s">
         <v>273</v>
       </c>
       <c r="D74" s="3" t="s">
@@ -6023,7 +6095,7 @@
       <c r="B75" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C75" s="10" t="s">
+      <c r="C75" s="3" t="s">
         <v>271</v>
       </c>
       <c r="D75" s="3" t="s">
@@ -6077,7 +6149,7 @@
       <c r="B76" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C76" s="10" t="s">
+      <c r="C76" s="3" t="s">
         <v>392</v>
       </c>
       <c r="D76" s="3" t="s">
@@ -6131,7 +6203,7 @@
       <c r="B77" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C77" s="10" t="s">
+      <c r="C77" s="3" t="s">
         <v>193</v>
       </c>
       <c r="D77" s="3" t="s">
@@ -6185,7 +6257,7 @@
       <c r="B78" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="C78" s="10" t="s">
+      <c r="C78" s="3" t="s">
         <v>277</v>
       </c>
       <c r="D78" s="3" t="s">
@@ -6239,7 +6311,7 @@
       <c r="B79" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="C79" s="10" t="s">
+      <c r="C79" s="3" t="s">
         <v>283</v>
       </c>
       <c r="D79" s="3" t="s">
@@ -6295,7 +6367,7 @@
       <c r="B80" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="C80" s="10" t="s">
+      <c r="C80" s="3" t="s">
         <v>112</v>
       </c>
       <c r="D80" s="3" t="s">
@@ -6348,7 +6420,7 @@
       <c r="B81" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C81" s="10" t="s">
+      <c r="C81" s="3" t="s">
         <v>83</v>
       </c>
       <c r="D81" s="3" t="s">
@@ -6404,7 +6476,7 @@
       <c r="B82" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C82" s="10" t="s">
+      <c r="C82" s="3" t="s">
         <v>83</v>
       </c>
       <c r="D82" s="3" t="s">
@@ -6459,7 +6531,7 @@
       <c r="B83" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C83" s="10" t="s">
+      <c r="C83" s="3" t="s">
         <v>289</v>
       </c>
       <c r="D83" s="3" t="s">
@@ -6515,7 +6587,7 @@
       <c r="B84" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C84" s="10" t="s">
+      <c r="C84" s="3" t="s">
         <v>94</v>
       </c>
       <c r="D84" s="3" t="s">
@@ -6571,7 +6643,7 @@
       <c r="B85" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C85" s="10" t="s">
+      <c r="C85" s="3" t="s">
         <v>395</v>
       </c>
       <c r="D85" s="3" t="s">
@@ -6625,7 +6697,7 @@
       <c r="B86" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C86" s="10" t="s">
+      <c r="C86" s="3" t="s">
         <v>286</v>
       </c>
       <c r="D86" s="3" t="s">
@@ -6681,7 +6753,7 @@
       <c r="B87" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C87" s="10" t="s">
+      <c r="C87" s="3" t="s">
         <v>290</v>
       </c>
       <c r="D87" s="3" t="s">
@@ -6735,7 +6807,7 @@
       <c r="B88" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="C88" s="10" t="s">
+      <c r="C88" s="3" t="s">
         <v>201</v>
       </c>
       <c r="D88" s="3" t="s">
@@ -6789,7 +6861,7 @@
       <c r="B89" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="C89" s="10" t="s">
+      <c r="C89" s="3" t="s">
         <v>292</v>
       </c>
       <c r="D89" s="3" t="s">
@@ -6845,7 +6917,7 @@
       <c r="B90" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="C90" s="10" t="s">
+      <c r="C90" s="3" t="s">
         <v>344</v>
       </c>
       <c r="D90" s="3" t="s">

</xml_diff>

<commit_message>
new specimen on morphosource
</commit_message>
<xml_diff>
--- a/Sample_data.xlsx
+++ b/Sample_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Document_UQAR\These\chapitre_2\Article\Repository\Raw_data_salamanders_modularity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C426552-BEF6-443A-B2B6-00BC895FFEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D72446C-CCFB-417F-A40A-4066CCABEE0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1400" uniqueCount="572">
   <si>
     <t>Family</t>
   </si>
@@ -997,9 +997,6 @@
     <t>Hydromantes platycephalus</t>
   </si>
   <si>
-    <t>Californa</t>
-  </si>
-  <si>
     <t>Inyo County</t>
   </si>
   <si>
@@ -1679,6 +1676,72 @@
   </si>
   <si>
     <t>https://www.morphosource.org/concern/media/000859442?locale=en</t>
+  </si>
+  <si>
+    <t>000859696</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859696?locale=en</t>
+  </si>
+  <si>
+    <t>000859710</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859710?locale=en</t>
+  </si>
+  <si>
+    <t>000859716</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859716?locale=en</t>
+  </si>
+  <si>
+    <t>000859723</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859723?locale=en</t>
+  </si>
+  <si>
+    <t>000859728</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859728?locale=en</t>
+  </si>
+  <si>
+    <t>000859742</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859742?locale=en</t>
+  </si>
+  <si>
+    <t>000859776</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859776?locale=en</t>
+  </si>
+  <si>
+    <t>000859786</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859786?locale=en</t>
+  </si>
+  <si>
+    <t>000859810</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859810?locale=en</t>
+  </si>
+  <si>
+    <t>000859801</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859801?locale=en</t>
+  </si>
+  <si>
+    <t>000859816</t>
+  </si>
+  <si>
+    <t>https://www.morphosource.org/concern/media/000859816?locale=en</t>
   </si>
 </sst>
 </file>
@@ -1717,18 +1780,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1743,7 +1800,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1766,9 +1823,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2026,7 +2080,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>3</v>
@@ -2068,10 +2122,10 @@
         <v>15</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2085,7 +2139,7 @@
         <v>108</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>19</v>
@@ -2123,10 +2177,10 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="9" t="s">
+        <v>526</v>
+      </c>
+      <c r="S2" t="s">
         <v>527</v>
-      </c>
-      <c r="S2" t="s">
-        <v>528</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2140,7 +2194,7 @@
         <v>120</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>49</v>
@@ -2182,7 +2236,7 @@
         <v>123</v>
       </c>
       <c r="R3" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2196,7 +2250,7 @@
         <v>124</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>49</v>
@@ -2238,7 +2292,7 @@
         <v>127</v>
       </c>
       <c r="R4" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2252,7 +2306,7 @@
         <v>113</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>19</v>
@@ -2261,10 +2315,10 @@
         <v>20</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
@@ -2298,7 +2352,7 @@
         <v>128</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>49</v>
@@ -2340,7 +2394,7 @@
         <v>21</v>
       </c>
       <c r="R6" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2354,7 +2408,7 @@
         <v>130</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>49</v>
@@ -2396,7 +2450,7 @@
         <v>134</v>
       </c>
       <c r="R7" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="8" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2410,7 +2464,7 @@
         <v>70</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>19</v>
@@ -2448,7 +2502,7 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2462,7 +2516,7 @@
         <v>301</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>19</v>
@@ -2498,10 +2552,10 @@
         <v>21</v>
       </c>
       <c r="R9" s="9" t="s">
+        <v>506</v>
+      </c>
+      <c r="S9" t="s">
         <v>507</v>
-      </c>
-      <c r="S9" t="s">
-        <v>508</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2515,7 +2569,7 @@
         <v>142</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>49</v>
@@ -2555,7 +2609,7 @@
         <v>21</v>
       </c>
       <c r="R10" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2569,7 +2623,7 @@
         <v>136</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>49</v>
@@ -2609,7 +2663,7 @@
         <v>62</v>
       </c>
       <c r="R11" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="12" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2623,7 +2677,7 @@
         <v>137</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>49</v>
@@ -2663,7 +2717,7 @@
         <v>141</v>
       </c>
       <c r="R12" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="13" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2677,7 +2731,7 @@
         <v>212</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>49</v>
@@ -2717,10 +2771,10 @@
         <v>21</v>
       </c>
       <c r="R13" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="S13" t="s">
         <v>523</v>
-      </c>
-      <c r="S13" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2734,7 +2788,7 @@
         <v>215</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>49</v>
@@ -2774,10 +2828,10 @@
         <v>21</v>
       </c>
       <c r="R14" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="S14" t="s">
         <v>525</v>
-      </c>
-      <c r="S14" t="s">
-        <v>526</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2791,7 +2845,7 @@
         <v>203</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>49</v>
@@ -2829,10 +2883,10 @@
       <c r="P15" s="3"/>
       <c r="Q15" s="3"/>
       <c r="R15" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="S15" t="s">
         <v>504</v>
-      </c>
-      <c r="S15" t="s">
-        <v>505</v>
       </c>
     </row>
     <row r="16" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2846,7 +2900,7 @@
         <v>203</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>49</v>
@@ -2884,10 +2938,10 @@
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
       <c r="R16" s="7" t="s">
+        <v>501</v>
+      </c>
+      <c r="S16" t="s">
         <v>502</v>
-      </c>
-      <c r="S16" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2898,10 +2952,10 @@
         <v>202</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>49</v>
@@ -2910,7 +2964,7 @@
         <v>25</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H17" s="3">
         <v>40080</v>
@@ -2929,22 +2983,22 @@
         <v>106</v>
       </c>
       <c r="N17" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="O17" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="O17" s="3" t="s">
+      <c r="P17" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="P17" s="3" t="s">
+      <c r="Q17" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="Q17" s="3" t="s">
-        <v>340</v>
-      </c>
       <c r="R17" s="7" t="s">
+        <v>499</v>
+      </c>
+      <c r="S17" t="s">
         <v>500</v>
-      </c>
-      <c r="S17" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2958,7 +3012,7 @@
         <v>235</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>49</v>
@@ -2998,10 +3052,10 @@
         <v>21</v>
       </c>
       <c r="R18" s="9" t="s">
+        <v>528</v>
+      </c>
+      <c r="S18" t="s">
         <v>529</v>
-      </c>
-      <c r="S18" t="s">
-        <v>530</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3015,7 +3069,7 @@
         <v>239</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>49</v>
@@ -3055,10 +3109,10 @@
         <v>21</v>
       </c>
       <c r="R19" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="S19" t="s">
         <v>531</v>
-      </c>
-      <c r="S19" t="s">
-        <v>532</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3072,7 +3126,7 @@
         <v>228</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>49</v>
@@ -3112,10 +3166,10 @@
         <v>21</v>
       </c>
       <c r="R20" s="9" t="s">
+        <v>532</v>
+      </c>
+      <c r="S20" t="s">
         <v>533</v>
-      </c>
-      <c r="S20" t="s">
-        <v>534</v>
       </c>
     </row>
     <row r="21" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3129,7 +3183,7 @@
         <v>243</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>49</v>
@@ -3171,10 +3225,10 @@
         <v>21</v>
       </c>
       <c r="R21" s="9" t="s">
+        <v>534</v>
+      </c>
+      <c r="S21" t="s">
         <v>535</v>
-      </c>
-      <c r="S21" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="22" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3184,11 +3238,11 @@
       <c r="B22" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="3" t="s">
         <v>225</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>49</v>
@@ -3230,10 +3284,10 @@
         <v>21</v>
       </c>
       <c r="R22" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="S22" t="s">
         <v>539</v>
-      </c>
-      <c r="S22" t="s">
-        <v>540</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3243,11 +3297,11 @@
       <c r="B23" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="3" t="s">
         <v>222</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>49</v>
@@ -3287,10 +3341,10 @@
         <v>21</v>
       </c>
       <c r="R23" s="9" t="s">
+        <v>536</v>
+      </c>
+      <c r="S23" t="s">
         <v>537</v>
-      </c>
-      <c r="S23" t="s">
-        <v>538</v>
       </c>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3300,11 +3354,11 @@
       <c r="B24" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="3" t="s">
         <v>218</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>49</v>
@@ -3346,10 +3400,10 @@
         <v>21</v>
       </c>
       <c r="R24" s="9" t="s">
+        <v>546</v>
+      </c>
+      <c r="S24" t="s">
         <v>547</v>
-      </c>
-      <c r="S24" t="s">
-        <v>548</v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3359,11 +3413,11 @@
       <c r="B25" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="3" t="s">
         <v>230</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>49</v>
@@ -3405,10 +3459,10 @@
         <v>21</v>
       </c>
       <c r="R25" s="9" t="s">
+        <v>542</v>
+      </c>
+      <c r="S25" t="s">
         <v>543</v>
-      </c>
-      <c r="S25" t="s">
-        <v>544</v>
       </c>
     </row>
     <row r="26" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3418,11 +3472,11 @@
       <c r="B26" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="3" t="s">
         <v>230</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>49</v>
@@ -3464,10 +3518,10 @@
         <v>21</v>
       </c>
       <c r="R26" s="9" t="s">
+        <v>544</v>
+      </c>
+      <c r="S26" t="s">
         <v>545</v>
-      </c>
-      <c r="S26" t="s">
-        <v>546</v>
       </c>
     </row>
     <row r="27" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3481,7 +3535,7 @@
         <v>230</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>49</v>
@@ -3523,10 +3577,10 @@
         <v>21</v>
       </c>
       <c r="R27" s="9" t="s">
+        <v>548</v>
+      </c>
+      <c r="S27" t="s">
         <v>549</v>
-      </c>
-      <c r="S27" t="s">
-        <v>550</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3536,11 +3590,11 @@
       <c r="B28" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="3" t="s">
         <v>246</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>49</v>
@@ -3580,10 +3634,10 @@
         <v>21</v>
       </c>
       <c r="R28" s="9" t="s">
+        <v>540</v>
+      </c>
+      <c r="S28" t="s">
         <v>541</v>
-      </c>
-      <c r="S28" t="s">
-        <v>542</v>
       </c>
     </row>
     <row r="29" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3597,7 +3651,7 @@
         <v>306</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>19</v>
@@ -3633,10 +3687,10 @@
         <v>21</v>
       </c>
       <c r="R29" s="9" t="s">
+        <v>508</v>
+      </c>
+      <c r="S29" t="s">
         <v>509</v>
-      </c>
-      <c r="S29" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="30" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3646,11 +3700,11 @@
       <c r="B30" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="10" t="s">
         <v>315</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>49</v>
@@ -3692,7 +3746,10 @@
         <v>21</v>
       </c>
       <c r="R30" s="9" t="s">
-        <v>506</v>
+        <v>550</v>
+      </c>
+      <c r="S30" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="31" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3706,7 +3763,7 @@
         <v>146</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>49</v>
@@ -3746,7 +3803,7 @@
         <v>21</v>
       </c>
       <c r="R31" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="32" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3756,11 +3813,11 @@
       <c r="B32" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="10" t="s">
         <v>318</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>49</v>
@@ -3802,7 +3859,10 @@
         <v>21</v>
       </c>
       <c r="R32" s="9" t="s">
-        <v>506</v>
+        <v>558</v>
+      </c>
+      <c r="S32" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="33" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3816,7 +3876,7 @@
         <v>147</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>49</v>
@@ -3856,7 +3916,7 @@
         <v>21</v>
       </c>
       <c r="R33" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="34" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3870,7 +3930,7 @@
         <v>148</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>49</v>
@@ -3910,7 +3970,7 @@
         <v>151</v>
       </c>
       <c r="R34" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="35" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3921,10 +3981,10 @@
         <v>63</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>49</v>
@@ -3933,7 +3993,7 @@
         <v>25</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H35" s="3">
         <v>15969</v>
@@ -3955,7 +4015,7 @@
         <v>37</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="P35" s="3" t="s">
         <v>21</v>
@@ -3964,10 +4024,10 @@
         <v>21</v>
       </c>
       <c r="R35" s="7" t="s">
+        <v>497</v>
+      </c>
+      <c r="S35" t="s">
         <v>498</v>
-      </c>
-      <c r="S35" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="36" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3981,7 +4041,7 @@
         <v>310</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>49</v>
@@ -4015,10 +4075,10 @@
         <v>21</v>
       </c>
       <c r="R36" s="9" t="s">
+        <v>510</v>
+      </c>
+      <c r="S36" t="s">
         <v>511</v>
-      </c>
-      <c r="S36" t="s">
-        <v>512</v>
       </c>
     </row>
     <row r="37" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4032,7 +4092,7 @@
         <v>153</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>49</v>
@@ -4072,7 +4132,7 @@
         <v>157</v>
       </c>
       <c r="R37" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="38" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4086,7 +4146,7 @@
         <v>158</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>49</v>
@@ -4126,7 +4186,7 @@
         <v>21</v>
       </c>
       <c r="R38" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="39" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4136,11 +4196,11 @@
       <c r="B39" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="10" t="s">
         <v>249</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>49</v>
@@ -4180,7 +4240,10 @@
         <v>21</v>
       </c>
       <c r="R39" s="9" t="s">
-        <v>506</v>
+        <v>552</v>
+      </c>
+      <c r="S39" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="40" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4194,7 +4257,7 @@
         <v>161</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>49</v>
@@ -4234,7 +4297,7 @@
         <v>164</v>
       </c>
       <c r="R40" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="41" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4244,11 +4307,11 @@
       <c r="B41" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="10" t="s">
         <v>252</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>49</v>
@@ -4288,7 +4351,10 @@
         <v>21</v>
       </c>
       <c r="R41" s="9" t="s">
-        <v>506</v>
+        <v>556</v>
+      </c>
+      <c r="S41" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="42" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4302,7 +4368,7 @@
         <v>166</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>49</v>
@@ -4342,7 +4408,7 @@
         <v>169</v>
       </c>
       <c r="R42" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="43" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4356,7 +4422,7 @@
         <v>171</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>49</v>
@@ -4398,7 +4464,7 @@
         <v>175</v>
       </c>
       <c r="R43" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="44" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4412,7 +4478,7 @@
         <v>74</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>49</v>
@@ -4450,10 +4516,10 @@
       <c r="P44" s="3"/>
       <c r="Q44" s="3"/>
       <c r="R44" s="7" t="s">
+        <v>493</v>
+      </c>
+      <c r="S44" t="s">
         <v>494</v>
-      </c>
-      <c r="S44" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="45" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4463,11 +4529,11 @@
       <c r="B45" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C45" s="10" t="s">
         <v>322</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>49</v>
@@ -4495,10 +4561,10 @@
         <v>32</v>
       </c>
       <c r="N45" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="O45" s="3" t="s">
         <v>323</v>
-      </c>
-      <c r="O45" s="3" t="s">
-        <v>324</v>
       </c>
       <c r="P45" s="3" t="s">
         <v>105</v>
@@ -4507,7 +4573,10 @@
         <v>21</v>
       </c>
       <c r="R45" s="9" t="s">
-        <v>506</v>
+        <v>564</v>
+      </c>
+      <c r="S45" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="46" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4517,11 +4586,11 @@
       <c r="B46" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" s="10" t="s">
         <v>255</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>49</v>
@@ -4563,7 +4632,10 @@
         <v>21</v>
       </c>
       <c r="R46" s="9" t="s">
-        <v>506</v>
+        <v>562</v>
+      </c>
+      <c r="S46" t="s">
+        <v>563</v>
       </c>
     </row>
     <row r="47" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4577,7 +4649,7 @@
         <v>312</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>49</v>
@@ -4611,10 +4683,10 @@
         <v>21</v>
       </c>
       <c r="R47" s="9" t="s">
+        <v>512</v>
+      </c>
+      <c r="S47" t="s">
         <v>513</v>
-      </c>
-      <c r="S47" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="48" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4624,11 +4696,11 @@
       <c r="B48" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C48" s="3" t="s">
-        <v>387</v>
+      <c r="C48" s="10" t="s">
+        <v>386</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>49</v>
@@ -4655,22 +4727,25 @@
         <v>27</v>
       </c>
       <c r="M48" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="N48" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="N48" s="3" t="s">
+      <c r="O48" s="3" t="s">
         <v>389</v>
       </c>
-      <c r="O48" s="3" t="s">
+      <c r="P48" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="P48" s="3" t="s">
-        <v>391</v>
-      </c>
       <c r="Q48" s="3" t="s">
         <v>21</v>
       </c>
       <c r="R48" s="9" t="s">
-        <v>506</v>
+        <v>570</v>
+      </c>
+      <c r="S48" t="s">
+        <v>571</v>
       </c>
     </row>
     <row r="49" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4680,11 +4755,11 @@
       <c r="B49" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="C49" s="10" t="s">
         <v>259</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>49</v>
@@ -4726,7 +4801,10 @@
         <v>21</v>
       </c>
       <c r="R49" s="9" t="s">
-        <v>506</v>
+        <v>566</v>
+      </c>
+      <c r="S49" t="s">
+        <v>567</v>
       </c>
     </row>
     <row r="50" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4736,11 +4814,11 @@
       <c r="B50" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C50" s="3" t="s">
-        <v>396</v>
+      <c r="C50" s="10" t="s">
+        <v>395</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>49</v>
@@ -4770,19 +4848,22 @@
         <v>106</v>
       </c>
       <c r="N50" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="O50" s="3" t="s">
         <v>397</v>
       </c>
-      <c r="O50" s="3" t="s">
+      <c r="P50" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q50" s="3" t="s">
         <v>398</v>
       </c>
-      <c r="P50" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="Q50" s="3" t="s">
-        <v>399</v>
-      </c>
       <c r="R50" s="9" t="s">
-        <v>506</v>
+        <v>568</v>
+      </c>
+      <c r="S50" t="s">
+        <v>569</v>
       </c>
     </row>
     <row r="51" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4796,7 +4877,7 @@
         <v>177</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>49</v>
@@ -4836,7 +4917,7 @@
         <v>21</v>
       </c>
       <c r="R51" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="52" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4850,7 +4931,7 @@
         <v>39</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>49</v>
@@ -4888,10 +4969,10 @@
       <c r="P52" s="3"/>
       <c r="Q52" s="3"/>
       <c r="R52" s="8" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="S52" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="53" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4905,7 +4986,7 @@
         <v>39</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>49</v>
@@ -4943,10 +5024,10 @@
       <c r="P53" s="3"/>
       <c r="Q53" s="3"/>
       <c r="R53" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="S53" t="s">
         <v>492</v>
-      </c>
-      <c r="S53" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="54" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4956,11 +5037,11 @@
       <c r="B54" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="10" t="s">
         <v>39</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E54" s="3" t="s">
         <v>49</v>
@@ -5002,7 +5083,10 @@
         <v>21</v>
       </c>
       <c r="R54" s="9" t="s">
-        <v>506</v>
+        <v>560</v>
+      </c>
+      <c r="S54" t="s">
+        <v>561</v>
       </c>
     </row>
     <row r="55" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5016,7 +5100,7 @@
         <v>78</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>49</v>
@@ -5054,10 +5138,10 @@
       <c r="P55" s="3"/>
       <c r="Q55" s="3"/>
       <c r="R55" s="7" t="s">
+        <v>487</v>
+      </c>
+      <c r="S55" t="s">
         <v>488</v>
-      </c>
-      <c r="S55" t="s">
-        <v>489</v>
       </c>
     </row>
     <row r="56" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5065,13 +5149,13 @@
         <v>65</v>
       </c>
       <c r="B56" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="C56" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="C56" s="3" t="s">
-        <v>326</v>
-      </c>
       <c r="D56" s="3" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="E56" s="3" t="s">
         <v>49</v>
@@ -5096,22 +5180,22 @@
       </c>
       <c r="L56" s="3"/>
       <c r="M56" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="N56" s="3" t="s">
         <v>327</v>
       </c>
-      <c r="N56" s="3" t="s">
+      <c r="O56" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="O56" s="3" t="s">
+      <c r="P56" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="P56" s="3" t="s">
-        <v>330</v>
-      </c>
       <c r="Q56" s="3" t="s">
         <v>21</v>
       </c>
       <c r="R56" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="57" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5121,11 +5205,11 @@
       <c r="B57" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C57" s="3" t="s">
+      <c r="C57" s="10" t="s">
         <v>18</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="E57" s="3" t="s">
         <v>19</v>
@@ -5134,10 +5218,10 @@
         <v>25</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="I57" s="3">
         <v>267</v>
@@ -5167,7 +5251,7 @@
         <v>21</v>
       </c>
       <c r="R57" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="58" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5177,11 +5261,11 @@
       <c r="B58" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="C58" s="10" t="s">
         <v>18</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>19</v>
@@ -5190,10 +5274,10 @@
         <v>25</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="I58" s="3">
         <v>239</v>
@@ -5223,7 +5307,7 @@
         <v>21</v>
       </c>
       <c r="R58" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="59" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5231,13 +5315,13 @@
         <v>65</v>
       </c>
       <c r="B59" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="C59" s="10" t="s">
         <v>352</v>
       </c>
-      <c r="C59" s="3" t="s">
-        <v>353</v>
-      </c>
       <c r="D59" s="3" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>49</v>
@@ -5246,10 +5330,10 @@
         <v>25</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="I59" s="3">
         <v>8.1</v>
@@ -5279,7 +5363,7 @@
         <v>21</v>
       </c>
       <c r="R59" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="60" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5287,13 +5371,13 @@
         <v>65</v>
       </c>
       <c r="B60" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="C60" s="10" t="s">
         <v>352</v>
       </c>
-      <c r="C60" s="3" t="s">
-        <v>353</v>
-      </c>
       <c r="D60" s="3" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="E60" s="3" t="s">
         <v>49</v>
@@ -5302,10 +5386,10 @@
         <v>25</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I60" s="3">
         <v>7.6</v>
@@ -5335,7 +5419,7 @@
         <v>21</v>
       </c>
       <c r="R60" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="61" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5349,7 +5433,7 @@
         <v>266</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>49</v>
@@ -5389,7 +5473,7 @@
         <v>21</v>
       </c>
       <c r="R61" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="62" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5403,7 +5487,7 @@
         <v>80</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>49</v>
@@ -5441,10 +5525,10 @@
       <c r="P62" s="3"/>
       <c r="Q62" s="3"/>
       <c r="R62" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="S62" t="s">
         <v>490</v>
-      </c>
-      <c r="S62" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="63" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5458,7 +5542,7 @@
         <v>267</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="E63" s="3" t="s">
         <v>49</v>
@@ -5498,7 +5582,7 @@
         <v>21</v>
       </c>
       <c r="R63" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="64" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5509,10 +5593,10 @@
         <v>52</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>49</v>
@@ -5542,19 +5626,19 @@
         <v>260</v>
       </c>
       <c r="N64" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="O64" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="O64" s="3" t="s">
+      <c r="P64" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q64" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="P64" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="Q64" s="3" t="s">
-        <v>334</v>
-      </c>
       <c r="R64" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="65" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5564,11 +5648,11 @@
       <c r="B65" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C65" s="10" t="s">
         <v>117</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>49</v>
@@ -5610,7 +5694,10 @@
         <v>21</v>
       </c>
       <c r="R65" s="9" t="s">
-        <v>506</v>
+        <v>554</v>
+      </c>
+      <c r="S65" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="66" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5624,7 +5711,7 @@
         <v>102</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="E66" s="3" t="s">
         <v>49</v>
@@ -5666,7 +5753,7 @@
         <v>190</v>
       </c>
       <c r="R66" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="67" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5680,7 +5767,7 @@
         <v>184</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="E67" s="3" t="s">
         <v>49</v>
@@ -5720,7 +5807,7 @@
         <v>187</v>
       </c>
       <c r="R67" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="68" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5734,7 +5821,7 @@
         <v>182</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="E68" s="3" t="s">
         <v>49</v>
@@ -5774,7 +5861,7 @@
         <v>21</v>
       </c>
       <c r="R68" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="69" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5788,7 +5875,7 @@
         <v>178</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>49</v>
@@ -5828,7 +5915,7 @@
         <v>181</v>
       </c>
       <c r="R69" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="70" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5842,7 +5929,7 @@
         <v>296</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="E70" s="3" t="s">
         <v>49</v>
@@ -5876,10 +5963,10 @@
         <v>21</v>
       </c>
       <c r="R70" s="9" t="s">
+        <v>514</v>
+      </c>
+      <c r="S70" t="s">
         <v>515</v>
-      </c>
-      <c r="S70" t="s">
-        <v>516</v>
       </c>
     </row>
     <row r="71" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5893,7 +5980,7 @@
         <v>67</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="E71" s="3" t="s">
         <v>49</v>
@@ -5929,10 +6016,10 @@
         <v>21</v>
       </c>
       <c r="R71" s="9" t="s">
+        <v>516</v>
+      </c>
+      <c r="S71" t="s">
         <v>517</v>
-      </c>
-      <c r="S71" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="72" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5946,7 +6033,7 @@
         <v>67</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="E72" s="3" t="s">
         <v>49</v>
@@ -5982,10 +6069,10 @@
         <v>21</v>
       </c>
       <c r="R72" s="9" t="s">
+        <v>518</v>
+      </c>
+      <c r="S72" t="s">
         <v>519</v>
-      </c>
-      <c r="S72" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="73" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5999,7 +6086,7 @@
         <v>115</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="E73" s="3" t="s">
         <v>19</v>
@@ -6008,10 +6095,10 @@
         <v>20</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="I73" s="3"/>
       <c r="J73" s="3"/>
@@ -6045,7 +6132,7 @@
         <v>273</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E74" s="3" t="s">
         <v>49</v>
@@ -6085,7 +6172,7 @@
         <v>21</v>
       </c>
       <c r="R74" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="75" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6099,7 +6186,7 @@
         <v>271</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E75" s="3" t="s">
         <v>49</v>
@@ -6139,7 +6226,7 @@
         <v>21</v>
       </c>
       <c r="R75" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="76" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6150,10 +6237,10 @@
         <v>54</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>49</v>
@@ -6184,16 +6271,16 @@
         <v>92</v>
       </c>
       <c r="O76" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="P76" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="P76" s="3" t="s">
-        <v>394</v>
-      </c>
       <c r="Q76" s="3" t="s">
         <v>21</v>
       </c>
       <c r="R76" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="77" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6207,7 +6294,7 @@
         <v>193</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="E77" s="3" t="s">
         <v>49</v>
@@ -6247,7 +6334,7 @@
         <v>196</v>
       </c>
       <c r="R77" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="78" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6261,7 +6348,7 @@
         <v>277</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="E78" s="3" t="s">
         <v>49</v>
@@ -6301,7 +6388,7 @@
         <v>21</v>
       </c>
       <c r="R78" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="79" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6315,7 +6402,7 @@
         <v>283</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="E79" s="3" t="s">
         <v>49</v>
@@ -6357,7 +6444,7 @@
         <v>21</v>
       </c>
       <c r="R79" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="80" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6371,7 +6458,7 @@
         <v>112</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="E80" s="3" t="s">
         <v>19</v>
@@ -6407,10 +6494,10 @@
         <v>21</v>
       </c>
       <c r="R80" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="S80" t="s">
         <v>521</v>
-      </c>
-      <c r="S80" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="81" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6424,7 +6511,7 @@
         <v>83</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="E81" s="3" t="s">
         <v>49</v>
@@ -6466,7 +6553,7 @@
         <v>199</v>
       </c>
       <c r="R81" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="82" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6480,7 +6567,7 @@
         <v>83</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="E82" s="3" t="s">
         <v>49</v>
@@ -6518,10 +6605,10 @@
       <c r="P82" s="3"/>
       <c r="Q82" s="3"/>
       <c r="R82" s="7" t="s">
+        <v>485</v>
+      </c>
+      <c r="S82" t="s">
         <v>486</v>
-      </c>
-      <c r="S82" t="s">
-        <v>487</v>
       </c>
     </row>
     <row r="83" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6535,7 +6622,7 @@
         <v>289</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="E83" s="3" t="s">
         <v>49</v>
@@ -6577,7 +6664,7 @@
         <v>21</v>
       </c>
       <c r="R83" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="84" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6591,7 +6678,7 @@
         <v>94</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="E84" s="3" t="s">
         <v>49</v>
@@ -6633,7 +6720,7 @@
         <v>21</v>
       </c>
       <c r="R84" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="85" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6644,10 +6731,10 @@
         <v>93</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="E85" s="3" t="s">
         <v>49</v>
@@ -6687,7 +6774,7 @@
         <v>21</v>
       </c>
       <c r="R85" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="86" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6701,7 +6788,7 @@
         <v>286</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>49</v>
@@ -6743,7 +6830,7 @@
         <v>21</v>
       </c>
       <c r="R86" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="87" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6757,7 +6844,7 @@
         <v>290</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="E87" s="3" t="s">
         <v>49</v>
@@ -6797,7 +6884,7 @@
         <v>21</v>
       </c>
       <c r="R87" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="88" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6811,7 +6898,7 @@
         <v>201</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="E88" s="3" t="s">
         <v>49</v>
@@ -6851,7 +6938,7 @@
         <v>21</v>
       </c>
       <c r="R88" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="89" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6865,7 +6952,7 @@
         <v>292</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>49</v>
@@ -6907,7 +6994,7 @@
         <v>21</v>
       </c>
       <c r="R89" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="90" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6915,13 +7002,13 @@
         <v>65</v>
       </c>
       <c r="B90" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="C90" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="C90" s="3" t="s">
-        <v>344</v>
-      </c>
       <c r="D90" s="3" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="E90" s="3" t="s">
         <v>49</v>
@@ -6930,7 +7017,7 @@
         <v>25</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H90" s="3">
         <v>35339</v>
@@ -6948,25 +7035,25 @@
         <v>27</v>
       </c>
       <c r="M90" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="N90" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="N90" s="3" t="s">
+      <c r="O90" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="O90" s="3" t="s">
+      <c r="P90" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="P90" s="3" t="s">
+      <c r="Q90" s="3" t="s">
         <v>348</v>
       </c>
-      <c r="Q90" s="3" t="s">
-        <v>349</v>
-      </c>
       <c r="R90" s="7" t="s">
+        <v>495</v>
+      </c>
+      <c r="S90" t="s">
         <v>496</v>
-      </c>
-      <c r="S90" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="91" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -7854,13 +7941,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>357</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7902,7 +7989,7 @@
         <v>304</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C4" s="2">
         <v>0</v>
@@ -8004,7 +8091,7 @@
         <v>33</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C10" s="2">
         <v>0</v>
@@ -8021,7 +8108,7 @@
         <v>65</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C11" s="2">
         <v>0</v>
@@ -8038,7 +8125,7 @@
         <v>65</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C12" s="2">
         <v>0</v>
@@ -8174,7 +8261,7 @@
         <v>65</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C20" s="2">
         <v>0</v>
@@ -8208,7 +8295,7 @@
         <v>65</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C22" s="2">
         <v>0</v>
@@ -8259,7 +8346,7 @@
         <v>33</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C25" s="2">
         <v>0</v>
@@ -8344,7 +8431,7 @@
         <v>33</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C30" s="2">
         <v>0</v>
@@ -8361,7 +8448,7 @@
         <v>33</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C31" s="2">
         <v>0</v>
@@ -8378,7 +8465,7 @@
         <v>65</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C32" s="2">
         <v>0</v>
@@ -8412,7 +8499,7 @@
         <v>51</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C34" s="2">
         <v>0</v>
@@ -8429,7 +8516,7 @@
         <v>65</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C35" s="2">
         <v>1</v>
@@ -8446,7 +8533,7 @@
         <v>65</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C36" s="2">
         <v>0</v>
@@ -8480,7 +8567,7 @@
         <v>65</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C38" s="2">
         <v>1</v>
@@ -8497,7 +8584,7 @@
         <v>65</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C39" s="2">
         <v>0</v>
@@ -8531,7 +8618,7 @@
         <v>33</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C41" s="2">
         <v>0</v>
@@ -8565,7 +8652,7 @@
         <v>65</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C43" s="2">
         <v>0</v>
@@ -8599,7 +8686,7 @@
         <v>51</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C45" s="2">
         <v>0</v>
@@ -8633,7 +8720,7 @@
         <v>51</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C47" s="2">
         <v>0</v>
@@ -8650,7 +8737,7 @@
         <v>65</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C48" s="2">
         <v>2</v>
@@ -8667,7 +8754,7 @@
         <v>33</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C49" s="2">
         <v>0</v>
@@ -8684,7 +8771,7 @@
         <v>33</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C50" s="2">
         <v>0</v>
@@ -8718,7 +8805,7 @@
         <v>65</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C52" s="2">
         <v>0</v>
@@ -8735,7 +8822,7 @@
         <v>16</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C53" s="2">
         <v>0</v>
@@ -8786,7 +8873,7 @@
         <v>51</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C56" s="2">
         <v>1</v>
@@ -8803,7 +8890,7 @@
         <v>33</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C57" s="2">
         <v>0</v>
@@ -8820,7 +8907,7 @@
         <v>51</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C58" s="2">
         <v>0</v>
@@ -8888,7 +8975,7 @@
         <v>65</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C62" s="2">
         <v>0</v>
@@ -8922,7 +9009,7 @@
         <v>33</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C64" s="2">
         <v>0</v>
@@ -8990,7 +9077,7 @@
         <v>65</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C68" s="2">
         <v>5</v>
@@ -9007,7 +9094,7 @@
         <v>33</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C69" s="2">
         <v>0</v>
@@ -9029,7 +9116,7 @@
     <row r="71" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
       <c r="B71" s="1" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C71" s="2">
         <f t="shared" ref="C71:E71" si="0">SUM(C2:C69)</f>

</xml_diff>